<commit_message>
Haftalik bulten 25.02.2026 (1 gun, toplam 31 mac)
</commit_message>
<xml_diff>
--- a/guncel_json/25022026.xlsx
+++ b/guncel_json/25022026.xlsx
@@ -1,18 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AyberkEylülKemal\Desktop\TahminApp\oddsy-data\guncel_json\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9084"/>
   </bookViews>
   <sheets>
     <sheet name="Tüm Veriler" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="407">
   <si>
     <t>Id</t>
   </si>
@@ -35,12 +42,6 @@
     <t>Dep</t>
   </si>
   <si>
-    <t>IYSkor</t>
-  </si>
-  <si>
-    <t>MSSkor</t>
-  </si>
-  <si>
     <t>MS1 A</t>
   </si>
   <si>
@@ -1233,28 +1234,34 @@
   </si>
   <si>
     <t>3.80</t>
+  </si>
+  <si>
+    <t>Featured</t>
+  </si>
+  <si>
+    <t>Ready</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="MM/dd/yyyy"/>
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000" tint="0"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFFFFFF" tint="0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -1267,17 +1274,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCDC610" tint="0"/>
+        <fgColor rgb="FFCDC610"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF008080" tint="0"/>
+        <fgColor rgb="FF008080"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEF981C" tint="0"/>
+        <fgColor rgb="FFEF981C"/>
       </patternFill>
     </fill>
   </fills>
@@ -1291,29 +1298,29 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" xfId="0"/>
-    <xf numFmtId="0" applyNumberFormat="0" fontId="0"/>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="3" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="4" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" applyNumberFormat="0" fontId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" applyNumberFormat="1" fontId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1321,6 +1328,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1328,474 +1344,711 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:HS32">
   <autoFilter ref="A1:HS32"/>
   <tableColumns count="227">
-    <tableColumn id="1" name="Id" totalsRowFunction="none"/>
-    <tableColumn id="2" name="BitmisMac" totalsRowFunction="none"/>
-    <tableColumn id="3" name="MatchCode" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Lig" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Tarih" totalsRowFunction="none"/>
-    <tableColumn id="6" name="Ev" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Dep" totalsRowFunction="none"/>
-    <tableColumn id="8" name="IYSkor" totalsRowFunction="none"/>
-    <tableColumn id="9" name="MSSkor" totalsRowFunction="none"/>
-    <tableColumn id="10" name="MS1 A" totalsRowFunction="none"/>
-    <tableColumn id="11" name="MS1 K" totalsRowFunction="none"/>
-    <tableColumn id="12" name="MS0 A" totalsRowFunction="none"/>
-    <tableColumn id="13" name="MS0 K" totalsRowFunction="none"/>
-    <tableColumn id="14" name="MS2 A" totalsRowFunction="none"/>
-    <tableColumn id="15" name="MS2 K" totalsRowFunction="none"/>
-    <tableColumn id="16" name="IY1 A" totalsRowFunction="none"/>
-    <tableColumn id="17" name="IY1 K" totalsRowFunction="none"/>
-    <tableColumn id="18" name="IY0 A" totalsRowFunction="none"/>
-    <tableColumn id="19" name="IY0 K" totalsRowFunction="none"/>
-    <tableColumn id="20" name="IY2 A" totalsRowFunction="none"/>
-    <tableColumn id="21" name="IY2 K" totalsRowFunction="none"/>
-    <tableColumn id="22" name="IIY1 A" totalsRowFunction="none"/>
-    <tableColumn id="23" name="IIY1 K" totalsRowFunction="none"/>
-    <tableColumn id="24" name="IIY0 A" totalsRowFunction="none"/>
-    <tableColumn id="25" name="IIY0 K" totalsRowFunction="none"/>
-    <tableColumn id="26" name="IIY2 A" totalsRowFunction="none"/>
-    <tableColumn id="27" name="IIY2 K" totalsRowFunction="none"/>
-    <tableColumn id="28" name="CS10 A" totalsRowFunction="none"/>
-    <tableColumn id="29" name="CS10 K" totalsRowFunction="none"/>
-    <tableColumn id="30" name="CS12 A" totalsRowFunction="none"/>
-    <tableColumn id="31" name="CS12 K" totalsRowFunction="none"/>
-    <tableColumn id="32" name="CS02 A" totalsRowFunction="none"/>
-    <tableColumn id="33" name="CS02 K" totalsRowFunction="none"/>
-    <tableColumn id="34" name="IYCS10 A" totalsRowFunction="none"/>
-    <tableColumn id="35" name="IYCS10 K" totalsRowFunction="none"/>
-    <tableColumn id="36" name="IYCS12 A" totalsRowFunction="none"/>
-    <tableColumn id="37" name="IYCS12 K" totalsRowFunction="none"/>
-    <tableColumn id="38" name="IYCS02 A" totalsRowFunction="none"/>
-    <tableColumn id="39" name="IYCS02 K" totalsRowFunction="none"/>
-    <tableColumn id="40" name="KGVAR A" totalsRowFunction="none"/>
-    <tableColumn id="41" name="KGVAR K" totalsRowFunction="none"/>
-    <tableColumn id="42" name="KGYOK A" totalsRowFunction="none"/>
-    <tableColumn id="43" name="KGYOK K" totalsRowFunction="none"/>
-    <tableColumn id="44" name="IY KGVAR A" totalsRowFunction="none"/>
-    <tableColumn id="45" name="IY KGVAR K" totalsRowFunction="none"/>
-    <tableColumn id="46" name="IY KGYOK A" totalsRowFunction="none"/>
-    <tableColumn id="47" name="IY KGYOK K" totalsRowFunction="none"/>
-    <tableColumn id="48" name="IIY KGVAR A" totalsRowFunction="none"/>
-    <tableColumn id="49" name="IIY KGVAR K" totalsRowFunction="none"/>
-    <tableColumn id="50" name="IIY KGYOK A" totalsRowFunction="none"/>
-    <tableColumn id="51" name="IIY KGYOK K" totalsRowFunction="none"/>
-    <tableColumn id="52" name="ALT05 A" totalsRowFunction="none"/>
-    <tableColumn id="53" name="ALT05 K" totalsRowFunction="none"/>
-    <tableColumn id="54" name="UST05 A" totalsRowFunction="none"/>
-    <tableColumn id="55" name="UST05 K" totalsRowFunction="none"/>
-    <tableColumn id="56" name="ALT15 A" totalsRowFunction="none"/>
-    <tableColumn id="57" name="ALT15 K" totalsRowFunction="none"/>
-    <tableColumn id="58" name="UST15 A" totalsRowFunction="none"/>
-    <tableColumn id="59" name="UST15 K" totalsRowFunction="none"/>
-    <tableColumn id="60" name="ALT25 A" totalsRowFunction="none"/>
-    <tableColumn id="61" name="ALT25 K" totalsRowFunction="none"/>
-    <tableColumn id="62" name="UST25 A" totalsRowFunction="none"/>
-    <tableColumn id="63" name="UST25 K" totalsRowFunction="none"/>
-    <tableColumn id="64" name="ALT35 A" totalsRowFunction="none"/>
-    <tableColumn id="65" name="ALT35 K" totalsRowFunction="none"/>
-    <tableColumn id="66" name="UST35 A" totalsRowFunction="none"/>
-    <tableColumn id="67" name="UST35 K" totalsRowFunction="none"/>
-    <tableColumn id="68" name="ALT45 A" totalsRowFunction="none"/>
-    <tableColumn id="69" name="ALT45 K" totalsRowFunction="none"/>
-    <tableColumn id="70" name="UST45 A" totalsRowFunction="none"/>
-    <tableColumn id="71" name="UST45 K" totalsRowFunction="none"/>
-    <tableColumn id="72" name="ALT55 A" totalsRowFunction="none"/>
-    <tableColumn id="73" name="ALT55 K" totalsRowFunction="none"/>
-    <tableColumn id="74" name="UST55 A" totalsRowFunction="none"/>
-    <tableColumn id="75" name="UST55 K" totalsRowFunction="none"/>
-    <tableColumn id="76" name="ALT65 A" totalsRowFunction="none"/>
-    <tableColumn id="77" name="ALT65 K" totalsRowFunction="none"/>
-    <tableColumn id="78" name="UST65 A" totalsRowFunction="none"/>
-    <tableColumn id="79" name="UST65 K" totalsRowFunction="none"/>
-    <tableColumn id="80" name="ALT75 A" totalsRowFunction="none"/>
-    <tableColumn id="81" name="ALT75 K" totalsRowFunction="none"/>
-    <tableColumn id="82" name="UST75 A" totalsRowFunction="none"/>
-    <tableColumn id="83" name="UST75 K" totalsRowFunction="none"/>
-    <tableColumn id="84" name="ALT85 A" totalsRowFunction="none"/>
-    <tableColumn id="85" name="ALT85 K" totalsRowFunction="none"/>
-    <tableColumn id="86" name="UST85 A" totalsRowFunction="none"/>
-    <tableColumn id="87" name="UST85 K" totalsRowFunction="none"/>
-    <tableColumn id="88" name="IYALT05 A" totalsRowFunction="none"/>
-    <tableColumn id="89" name="IYALT05 K" totalsRowFunction="none"/>
-    <tableColumn id="90" name="IYUST05 A" totalsRowFunction="none"/>
-    <tableColumn id="91" name="IYUST05 K" totalsRowFunction="none"/>
-    <tableColumn id="92" name="IYALT15 A" totalsRowFunction="none"/>
-    <tableColumn id="93" name="IYALT15 K" totalsRowFunction="none"/>
-    <tableColumn id="94" name="IYUST15 A" totalsRowFunction="none"/>
-    <tableColumn id="95" name="IYUST15 K" totalsRowFunction="none"/>
-    <tableColumn id="96" name="IYALT25 A" totalsRowFunction="none"/>
-    <tableColumn id="97" name="IYALT25 K" totalsRowFunction="none"/>
-    <tableColumn id="98" name="IYUST25 A" totalsRowFunction="none"/>
-    <tableColumn id="99" name="IYUST25 K" totalsRowFunction="none"/>
-    <tableColumn id="100" name="IYALT35 A" totalsRowFunction="none"/>
-    <tableColumn id="101" name="IYALT35 K" totalsRowFunction="none"/>
-    <tableColumn id="102" name="IYUST35 A" totalsRowFunction="none"/>
-    <tableColumn id="103" name="IYUST35 K" totalsRowFunction="none"/>
-    <tableColumn id="104" name="IYALT45 A" totalsRowFunction="none"/>
-    <tableColumn id="105" name="IYALT45 K" totalsRowFunction="none"/>
-    <tableColumn id="106" name="IYUST45 A" totalsRowFunction="none"/>
-    <tableColumn id="107" name="IYUST45 K" totalsRowFunction="none"/>
-    <tableColumn id="108" name="IYMS 1E1 A" totalsRowFunction="none"/>
-    <tableColumn id="109" name="IYMS 1E1 K" totalsRowFunction="none"/>
-    <tableColumn id="110" name="IYMS 1E0 A" totalsRowFunction="none"/>
-    <tableColumn id="111" name="IYMS 1E0 K" totalsRowFunction="none"/>
-    <tableColumn id="112" name="IYMS 1E2 A" totalsRowFunction="none"/>
-    <tableColumn id="113" name="IYMS 1E2 K" totalsRowFunction="none"/>
-    <tableColumn id="114" name="IYMS 0E1 A" totalsRowFunction="none"/>
-    <tableColumn id="115" name="IYMS 0E1 K" totalsRowFunction="none"/>
-    <tableColumn id="116" name="IYMS 0E0 A" totalsRowFunction="none"/>
-    <tableColumn id="117" name="IYMS 0E0 K" totalsRowFunction="none"/>
-    <tableColumn id="118" name="IYMS 0E2 A" totalsRowFunction="none"/>
-    <tableColumn id="119" name="IYMS 0E2 K" totalsRowFunction="none"/>
-    <tableColumn id="120" name="IYMS 2E1 A" totalsRowFunction="none"/>
-    <tableColumn id="121" name="IYMS 2E1 K" totalsRowFunction="none"/>
-    <tableColumn id="122" name="IYMS 2E0 A" totalsRowFunction="none"/>
-    <tableColumn id="123" name="IYMS 2E0 K" totalsRowFunction="none"/>
-    <tableColumn id="124" name="IYMS 2E2 A" totalsRowFunction="none"/>
-    <tableColumn id="125" name="IYMS 2E2 K" totalsRowFunction="none"/>
-    <tableColumn id="126" name="Score A10" totalsRowFunction="none"/>
-    <tableColumn id="127" name="Score K10" totalsRowFunction="none"/>
-    <tableColumn id="128" name="Score A20" totalsRowFunction="none"/>
-    <tableColumn id="129" name="Score K20" totalsRowFunction="none"/>
-    <tableColumn id="130" name="Score A30" totalsRowFunction="none"/>
-    <tableColumn id="131" name="Score K30" totalsRowFunction="none"/>
-    <tableColumn id="132" name="Score A40" totalsRowFunction="none"/>
-    <tableColumn id="133" name="Score K40" totalsRowFunction="none"/>
-    <tableColumn id="134" name="Score A50" totalsRowFunction="none"/>
-    <tableColumn id="135" name="Score K50" totalsRowFunction="none"/>
-    <tableColumn id="136" name="Score A60" totalsRowFunction="none"/>
-    <tableColumn id="137" name="Score K60" totalsRowFunction="none"/>
-    <tableColumn id="138" name="Score A70" totalsRowFunction="none"/>
-    <tableColumn id="139" name="Score K70" totalsRowFunction="none"/>
-    <tableColumn id="140" name="Score A21" totalsRowFunction="none"/>
-    <tableColumn id="141" name="Score K21" totalsRowFunction="none"/>
-    <tableColumn id="142" name="Score A31" totalsRowFunction="none"/>
-    <tableColumn id="143" name="Score K31" totalsRowFunction="none"/>
-    <tableColumn id="144" name="Score A41" totalsRowFunction="none"/>
-    <tableColumn id="145" name="Score K41" totalsRowFunction="none"/>
-    <tableColumn id="146" name="Score A51" totalsRowFunction="none"/>
-    <tableColumn id="147" name="Score K51" totalsRowFunction="none"/>
-    <tableColumn id="148" name="Score A61" totalsRowFunction="none"/>
-    <tableColumn id="149" name="Score K61" totalsRowFunction="none"/>
-    <tableColumn id="150" name="Score A32" totalsRowFunction="none"/>
-    <tableColumn id="151" name="Score K32" totalsRowFunction="none"/>
-    <tableColumn id="152" name="Score A42" totalsRowFunction="none"/>
-    <tableColumn id="153" name="Score K42" totalsRowFunction="none"/>
-    <tableColumn id="154" name="Score A52" totalsRowFunction="none"/>
-    <tableColumn id="155" name="Score K52" totalsRowFunction="none"/>
-    <tableColumn id="156" name="Score A43" totalsRowFunction="none"/>
-    <tableColumn id="157" name="Score K43" totalsRowFunction="none"/>
-    <tableColumn id="158" name="Score A00" totalsRowFunction="none"/>
-    <tableColumn id="159" name="Score K00" totalsRowFunction="none"/>
-    <tableColumn id="160" name="Score A11" totalsRowFunction="none"/>
-    <tableColumn id="161" name="Score K11" totalsRowFunction="none"/>
-    <tableColumn id="162" name="Score A22" totalsRowFunction="none"/>
-    <tableColumn id="163" name="Score K22" totalsRowFunction="none"/>
-    <tableColumn id="164" name="Score A33" totalsRowFunction="none"/>
-    <tableColumn id="165" name="Score K33" totalsRowFunction="none"/>
-    <tableColumn id="166" name="Score A01" totalsRowFunction="none"/>
-    <tableColumn id="167" name="Score K01" totalsRowFunction="none"/>
-    <tableColumn id="168" name="Score A02" totalsRowFunction="none"/>
-    <tableColumn id="169" name="Score K02" totalsRowFunction="none"/>
-    <tableColumn id="170" name="Score A03" totalsRowFunction="none"/>
-    <tableColumn id="171" name="Score K03" totalsRowFunction="none"/>
-    <tableColumn id="172" name="Score A04" totalsRowFunction="none"/>
-    <tableColumn id="173" name="Score K04" totalsRowFunction="none"/>
-    <tableColumn id="174" name="Score A05" totalsRowFunction="none"/>
-    <tableColumn id="175" name="Score K05" totalsRowFunction="none"/>
-    <tableColumn id="176" name="Score A06" totalsRowFunction="none"/>
-    <tableColumn id="177" name="Score K06" totalsRowFunction="none"/>
-    <tableColumn id="178" name="Score A07" totalsRowFunction="none"/>
-    <tableColumn id="179" name="Score K07" totalsRowFunction="none"/>
-    <tableColumn id="180" name="Score A12" totalsRowFunction="none"/>
-    <tableColumn id="181" name="Score K12" totalsRowFunction="none"/>
-    <tableColumn id="182" name="Score A13" totalsRowFunction="none"/>
-    <tableColumn id="183" name="Score K13" totalsRowFunction="none"/>
-    <tableColumn id="184" name="Score A14" totalsRowFunction="none"/>
-    <tableColumn id="185" name="Score K14" totalsRowFunction="none"/>
-    <tableColumn id="186" name="Score A15" totalsRowFunction="none"/>
-    <tableColumn id="187" name="Score K15" totalsRowFunction="none"/>
-    <tableColumn id="188" name="Score A16" totalsRowFunction="none"/>
-    <tableColumn id="189" name="Score K16" totalsRowFunction="none"/>
-    <tableColumn id="190" name="Score A23" totalsRowFunction="none"/>
-    <tableColumn id="191" name="Score K23" totalsRowFunction="none"/>
-    <tableColumn id="192" name="Score A24" totalsRowFunction="none"/>
-    <tableColumn id="193" name="Score K24" totalsRowFunction="none"/>
-    <tableColumn id="194" name="Score A25" totalsRowFunction="none"/>
-    <tableColumn id="195" name="Score K25" totalsRowFunction="none"/>
-    <tableColumn id="196" name="Score A34" totalsRowFunction="none"/>
-    <tableColumn id="197" name="Score K34" totalsRowFunction="none"/>
-    <tableColumn id="198" name="IYScore A10" totalsRowFunction="none"/>
-    <tableColumn id="199" name="IYScore K10" totalsRowFunction="none"/>
-    <tableColumn id="200" name="IYScore A20" totalsRowFunction="none"/>
-    <tableColumn id="201" name="IYScore K20" totalsRowFunction="none"/>
-    <tableColumn id="202" name="IYScore A30" totalsRowFunction="none"/>
-    <tableColumn id="203" name="IYScore K30" totalsRowFunction="none"/>
-    <tableColumn id="204" name="IYScore A40" totalsRowFunction="none"/>
-    <tableColumn id="205" name="IYScore K40" totalsRowFunction="none"/>
-    <tableColumn id="206" name="IYScore A21" totalsRowFunction="none"/>
-    <tableColumn id="207" name="IYScore K21" totalsRowFunction="none"/>
-    <tableColumn id="208" name="IYScore A31" totalsRowFunction="none"/>
-    <tableColumn id="209" name="IYScore K31" totalsRowFunction="none"/>
-    <tableColumn id="210" name="IYScore A00" totalsRowFunction="none"/>
-    <tableColumn id="211" name="IYScore K00" totalsRowFunction="none"/>
-    <tableColumn id="212" name="IYScore A11" totalsRowFunction="none"/>
-    <tableColumn id="213" name="IYScore K11" totalsRowFunction="none"/>
-    <tableColumn id="214" name="IYScore A22" totalsRowFunction="none"/>
-    <tableColumn id="215" name="IYScore K22" totalsRowFunction="none"/>
-    <tableColumn id="216" name="IYScore A01" totalsRowFunction="none"/>
-    <tableColumn id="217" name="IYScore K01" totalsRowFunction="none"/>
-    <tableColumn id="218" name="IYScore A02" totalsRowFunction="none"/>
-    <tableColumn id="219" name="IYScore K02" totalsRowFunction="none"/>
-    <tableColumn id="220" name="IYScore A03" totalsRowFunction="none"/>
-    <tableColumn id="221" name="IYScore K03" totalsRowFunction="none"/>
-    <tableColumn id="222" name="IYScore A04" totalsRowFunction="none"/>
-    <tableColumn id="223" name="IYScore K04" totalsRowFunction="none"/>
-    <tableColumn id="224" name="IYScore A12" totalsRowFunction="none"/>
-    <tableColumn id="225" name="IYScore K12" totalsRowFunction="none"/>
-    <tableColumn id="226" name="IYScore A13" totalsRowFunction="none"/>
-    <tableColumn id="227" name="IYScore K13" totalsRowFunction="none"/>
+    <tableColumn id="1" name="Id"/>
+    <tableColumn id="2" name="BitmisMac"/>
+    <tableColumn id="3" name="MatchCode"/>
+    <tableColumn id="4" name="Lig"/>
+    <tableColumn id="5" name="Tarih"/>
+    <tableColumn id="6" name="Ev"/>
+    <tableColumn id="7" name="Dep"/>
+    <tableColumn id="8" name="Featured"/>
+    <tableColumn id="9" name="Ready"/>
+    <tableColumn id="10" name="MS1 A"/>
+    <tableColumn id="11" name="MS1 K"/>
+    <tableColumn id="12" name="MS0 A"/>
+    <tableColumn id="13" name="MS0 K"/>
+    <tableColumn id="14" name="MS2 A"/>
+    <tableColumn id="15" name="MS2 K"/>
+    <tableColumn id="16" name="IY1 A"/>
+    <tableColumn id="17" name="IY1 K"/>
+    <tableColumn id="18" name="IY0 A"/>
+    <tableColumn id="19" name="IY0 K"/>
+    <tableColumn id="20" name="IY2 A"/>
+    <tableColumn id="21" name="IY2 K"/>
+    <tableColumn id="22" name="IIY1 A"/>
+    <tableColumn id="23" name="IIY1 K"/>
+    <tableColumn id="24" name="IIY0 A"/>
+    <tableColumn id="25" name="IIY0 K"/>
+    <tableColumn id="26" name="IIY2 A"/>
+    <tableColumn id="27" name="IIY2 K"/>
+    <tableColumn id="28" name="CS10 A"/>
+    <tableColumn id="29" name="CS10 K"/>
+    <tableColumn id="30" name="CS12 A"/>
+    <tableColumn id="31" name="CS12 K"/>
+    <tableColumn id="32" name="CS02 A"/>
+    <tableColumn id="33" name="CS02 K"/>
+    <tableColumn id="34" name="IYCS10 A"/>
+    <tableColumn id="35" name="IYCS10 K"/>
+    <tableColumn id="36" name="IYCS12 A"/>
+    <tableColumn id="37" name="IYCS12 K"/>
+    <tableColumn id="38" name="IYCS02 A"/>
+    <tableColumn id="39" name="IYCS02 K"/>
+    <tableColumn id="40" name="KGVAR A"/>
+    <tableColumn id="41" name="KGVAR K"/>
+    <tableColumn id="42" name="KGYOK A"/>
+    <tableColumn id="43" name="KGYOK K"/>
+    <tableColumn id="44" name="IY KGVAR A"/>
+    <tableColumn id="45" name="IY KGVAR K"/>
+    <tableColumn id="46" name="IY KGYOK A"/>
+    <tableColumn id="47" name="IY KGYOK K"/>
+    <tableColumn id="48" name="IIY KGVAR A"/>
+    <tableColumn id="49" name="IIY KGVAR K"/>
+    <tableColumn id="50" name="IIY KGYOK A"/>
+    <tableColumn id="51" name="IIY KGYOK K"/>
+    <tableColumn id="52" name="ALT05 A"/>
+    <tableColumn id="53" name="ALT05 K"/>
+    <tableColumn id="54" name="UST05 A"/>
+    <tableColumn id="55" name="UST05 K"/>
+    <tableColumn id="56" name="ALT15 A"/>
+    <tableColumn id="57" name="ALT15 K"/>
+    <tableColumn id="58" name="UST15 A"/>
+    <tableColumn id="59" name="UST15 K"/>
+    <tableColumn id="60" name="ALT25 A"/>
+    <tableColumn id="61" name="ALT25 K"/>
+    <tableColumn id="62" name="UST25 A"/>
+    <tableColumn id="63" name="UST25 K"/>
+    <tableColumn id="64" name="ALT35 A"/>
+    <tableColumn id="65" name="ALT35 K"/>
+    <tableColumn id="66" name="UST35 A"/>
+    <tableColumn id="67" name="UST35 K"/>
+    <tableColumn id="68" name="ALT45 A"/>
+    <tableColumn id="69" name="ALT45 K"/>
+    <tableColumn id="70" name="UST45 A"/>
+    <tableColumn id="71" name="UST45 K"/>
+    <tableColumn id="72" name="ALT55 A"/>
+    <tableColumn id="73" name="ALT55 K"/>
+    <tableColumn id="74" name="UST55 A"/>
+    <tableColumn id="75" name="UST55 K"/>
+    <tableColumn id="76" name="ALT65 A"/>
+    <tableColumn id="77" name="ALT65 K"/>
+    <tableColumn id="78" name="UST65 A"/>
+    <tableColumn id="79" name="UST65 K"/>
+    <tableColumn id="80" name="ALT75 A"/>
+    <tableColumn id="81" name="ALT75 K"/>
+    <tableColumn id="82" name="UST75 A"/>
+    <tableColumn id="83" name="UST75 K"/>
+    <tableColumn id="84" name="ALT85 A"/>
+    <tableColumn id="85" name="ALT85 K"/>
+    <tableColumn id="86" name="UST85 A"/>
+    <tableColumn id="87" name="UST85 K"/>
+    <tableColumn id="88" name="IYALT05 A"/>
+    <tableColumn id="89" name="IYALT05 K"/>
+    <tableColumn id="90" name="IYUST05 A"/>
+    <tableColumn id="91" name="IYUST05 K"/>
+    <tableColumn id="92" name="IYALT15 A"/>
+    <tableColumn id="93" name="IYALT15 K"/>
+    <tableColumn id="94" name="IYUST15 A"/>
+    <tableColumn id="95" name="IYUST15 K"/>
+    <tableColumn id="96" name="IYALT25 A"/>
+    <tableColumn id="97" name="IYALT25 K"/>
+    <tableColumn id="98" name="IYUST25 A"/>
+    <tableColumn id="99" name="IYUST25 K"/>
+    <tableColumn id="100" name="IYALT35 A"/>
+    <tableColumn id="101" name="IYALT35 K"/>
+    <tableColumn id="102" name="IYUST35 A"/>
+    <tableColumn id="103" name="IYUST35 K"/>
+    <tableColumn id="104" name="IYALT45 A"/>
+    <tableColumn id="105" name="IYALT45 K"/>
+    <tableColumn id="106" name="IYUST45 A"/>
+    <tableColumn id="107" name="IYUST45 K"/>
+    <tableColumn id="108" name="IYMS 1E1 A"/>
+    <tableColumn id="109" name="IYMS 1E1 K"/>
+    <tableColumn id="110" name="IYMS 1E0 A"/>
+    <tableColumn id="111" name="IYMS 1E0 K"/>
+    <tableColumn id="112" name="IYMS 1E2 A"/>
+    <tableColumn id="113" name="IYMS 1E2 K"/>
+    <tableColumn id="114" name="IYMS 0E1 A"/>
+    <tableColumn id="115" name="IYMS 0E1 K"/>
+    <tableColumn id="116" name="IYMS 0E0 A"/>
+    <tableColumn id="117" name="IYMS 0E0 K"/>
+    <tableColumn id="118" name="IYMS 0E2 A"/>
+    <tableColumn id="119" name="IYMS 0E2 K"/>
+    <tableColumn id="120" name="IYMS 2E1 A"/>
+    <tableColumn id="121" name="IYMS 2E1 K"/>
+    <tableColumn id="122" name="IYMS 2E0 A"/>
+    <tableColumn id="123" name="IYMS 2E0 K"/>
+    <tableColumn id="124" name="IYMS 2E2 A"/>
+    <tableColumn id="125" name="IYMS 2E2 K"/>
+    <tableColumn id="126" name="Score A10"/>
+    <tableColumn id="127" name="Score K10"/>
+    <tableColumn id="128" name="Score A20"/>
+    <tableColumn id="129" name="Score K20"/>
+    <tableColumn id="130" name="Score A30"/>
+    <tableColumn id="131" name="Score K30"/>
+    <tableColumn id="132" name="Score A40"/>
+    <tableColumn id="133" name="Score K40"/>
+    <tableColumn id="134" name="Score A50"/>
+    <tableColumn id="135" name="Score K50"/>
+    <tableColumn id="136" name="Score A60"/>
+    <tableColumn id="137" name="Score K60"/>
+    <tableColumn id="138" name="Score A70"/>
+    <tableColumn id="139" name="Score K70"/>
+    <tableColumn id="140" name="Score A21"/>
+    <tableColumn id="141" name="Score K21"/>
+    <tableColumn id="142" name="Score A31"/>
+    <tableColumn id="143" name="Score K31"/>
+    <tableColumn id="144" name="Score A41"/>
+    <tableColumn id="145" name="Score K41"/>
+    <tableColumn id="146" name="Score A51"/>
+    <tableColumn id="147" name="Score K51"/>
+    <tableColumn id="148" name="Score A61"/>
+    <tableColumn id="149" name="Score K61"/>
+    <tableColumn id="150" name="Score A32"/>
+    <tableColumn id="151" name="Score K32"/>
+    <tableColumn id="152" name="Score A42"/>
+    <tableColumn id="153" name="Score K42"/>
+    <tableColumn id="154" name="Score A52"/>
+    <tableColumn id="155" name="Score K52"/>
+    <tableColumn id="156" name="Score A43"/>
+    <tableColumn id="157" name="Score K43"/>
+    <tableColumn id="158" name="Score A00"/>
+    <tableColumn id="159" name="Score K00"/>
+    <tableColumn id="160" name="Score A11"/>
+    <tableColumn id="161" name="Score K11"/>
+    <tableColumn id="162" name="Score A22"/>
+    <tableColumn id="163" name="Score K22"/>
+    <tableColumn id="164" name="Score A33"/>
+    <tableColumn id="165" name="Score K33"/>
+    <tableColumn id="166" name="Score A01"/>
+    <tableColumn id="167" name="Score K01"/>
+    <tableColumn id="168" name="Score A02"/>
+    <tableColumn id="169" name="Score K02"/>
+    <tableColumn id="170" name="Score A03"/>
+    <tableColumn id="171" name="Score K03"/>
+    <tableColumn id="172" name="Score A04"/>
+    <tableColumn id="173" name="Score K04"/>
+    <tableColumn id="174" name="Score A05"/>
+    <tableColumn id="175" name="Score K05"/>
+    <tableColumn id="176" name="Score A06"/>
+    <tableColumn id="177" name="Score K06"/>
+    <tableColumn id="178" name="Score A07"/>
+    <tableColumn id="179" name="Score K07"/>
+    <tableColumn id="180" name="Score A12"/>
+    <tableColumn id="181" name="Score K12"/>
+    <tableColumn id="182" name="Score A13"/>
+    <tableColumn id="183" name="Score K13"/>
+    <tableColumn id="184" name="Score A14"/>
+    <tableColumn id="185" name="Score K14"/>
+    <tableColumn id="186" name="Score A15"/>
+    <tableColumn id="187" name="Score K15"/>
+    <tableColumn id="188" name="Score A16"/>
+    <tableColumn id="189" name="Score K16"/>
+    <tableColumn id="190" name="Score A23"/>
+    <tableColumn id="191" name="Score K23"/>
+    <tableColumn id="192" name="Score A24"/>
+    <tableColumn id="193" name="Score K24"/>
+    <tableColumn id="194" name="Score A25"/>
+    <tableColumn id="195" name="Score K25"/>
+    <tableColumn id="196" name="Score A34"/>
+    <tableColumn id="197" name="Score K34"/>
+    <tableColumn id="198" name="IYScore A10"/>
+    <tableColumn id="199" name="IYScore K10"/>
+    <tableColumn id="200" name="IYScore A20"/>
+    <tableColumn id="201" name="IYScore K20"/>
+    <tableColumn id="202" name="IYScore A30"/>
+    <tableColumn id="203" name="IYScore K30"/>
+    <tableColumn id="204" name="IYScore A40"/>
+    <tableColumn id="205" name="IYScore K40"/>
+    <tableColumn id="206" name="IYScore A21"/>
+    <tableColumn id="207" name="IYScore K21"/>
+    <tableColumn id="208" name="IYScore A31"/>
+    <tableColumn id="209" name="IYScore K31"/>
+    <tableColumn id="210" name="IYScore A00"/>
+    <tableColumn id="211" name="IYScore K00"/>
+    <tableColumn id="212" name="IYScore A11"/>
+    <tableColumn id="213" name="IYScore K11"/>
+    <tableColumn id="214" name="IYScore A22"/>
+    <tableColumn id="215" name="IYScore K22"/>
+    <tableColumn id="216" name="IYScore A01"/>
+    <tableColumn id="217" name="IYScore K01"/>
+    <tableColumn id="218" name="IYScore A02"/>
+    <tableColumn id="219" name="IYScore K02"/>
+    <tableColumn id="220" name="IYScore A03"/>
+    <tableColumn id="221" name="IYScore K03"/>
+    <tableColumn id="222" name="IYScore A04"/>
+    <tableColumn id="223" name="IYScore K04"/>
+    <tableColumn id="224" name="IYScore A12"/>
+    <tableColumn id="225" name="IYScore K12"/>
+    <tableColumn id="226" name="IYScore A13"/>
+    <tableColumn id="227" name="IYScore K13"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Teması">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4472C4"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName=""/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:HS32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1" style="4"/>
-    <col min="2" max="2" width="12.1948787144252" customWidth="1" style="4"/>
-    <col min="3" max="3" width="13.093129839216" customWidth="1" style="4"/>
-    <col min="4" max="4" width="29.4721287318638" customWidth="1" style="4"/>
-    <col min="5" max="5" width="10.5382559640067" customWidth="1" style="6"/>
-    <col min="6" max="6" width="25.0064479282924" customWidth="1" style="4"/>
-    <col min="7" max="7" width="19.225106375558" customWidth="1" style="4"/>
-    <col min="8" max="8" width="9.140625" customWidth="1" style="4"/>
-    <col min="9" max="9" width="9.64744567871094" customWidth="1" style="4"/>
-    <col min="10" max="10" width="9.140625" customWidth="1" style="4"/>
-    <col min="11" max="11" width="9.140625" customWidth="1" style="4"/>
-    <col min="12" max="12" width="9.140625" customWidth="1" style="4"/>
-    <col min="13" max="13" width="9.140625" customWidth="1" style="4"/>
-    <col min="14" max="14" width="9.140625" customWidth="1" style="4"/>
-    <col min="15" max="15" width="9.140625" customWidth="1" style="4"/>
-    <col min="16" max="16" width="9.140625" customWidth="1" style="4"/>
-    <col min="17" max="17" width="9.140625" customWidth="1" style="4"/>
-    <col min="18" max="18" width="9.140625" customWidth="1" style="4"/>
-    <col min="19" max="19" width="9.140625" customWidth="1" style="4"/>
-    <col min="20" max="20" width="9.140625" customWidth="1" style="4"/>
-    <col min="21" max="21" width="9.140625" customWidth="1" style="4"/>
-    <col min="22" max="22" width="9.140625" customWidth="1" style="4"/>
-    <col min="23" max="23" width="9.140625" customWidth="1" style="4"/>
-    <col min="24" max="24" width="9.140625" customWidth="1" style="4"/>
-    <col min="25" max="25" width="9.140625" customWidth="1" style="4"/>
-    <col min="26" max="26" width="9.140625" customWidth="1" style="4"/>
-    <col min="27" max="27" width="9.140625" customWidth="1" style="4"/>
-    <col min="28" max="28" width="9.140625" customWidth="1" style="4"/>
-    <col min="29" max="29" width="9.140625" customWidth="1" style="4"/>
-    <col min="30" max="30" width="9.140625" customWidth="1" style="4"/>
-    <col min="31" max="31" width="9.140625" customWidth="1" style="4"/>
-    <col min="32" max="32" width="9.140625" customWidth="1" style="4"/>
-    <col min="33" max="33" width="9.140625" customWidth="1" style="4"/>
-    <col min="34" max="34" width="10.6101499285017" customWidth="1" style="4"/>
-    <col min="35" max="35" width="10.4822671072824" customWidth="1" style="4"/>
-    <col min="36" max="36" width="10.6101499285017" customWidth="1" style="4"/>
-    <col min="37" max="37" width="10.4822671072824" customWidth="1" style="4"/>
-    <col min="38" max="38" width="10.6101499285017" customWidth="1" style="4"/>
-    <col min="39" max="39" width="10.4822671072824" customWidth="1" style="4"/>
-    <col min="40" max="40" width="10.8137403215681" customWidth="1" style="4"/>
-    <col min="41" max="41" width="10.6858564104353" customWidth="1" style="4"/>
-    <col min="42" max="42" width="10.7707715715681" customWidth="1" style="4"/>
-    <col min="43" max="43" width="10.6428876604353" customWidth="1" style="4"/>
-    <col min="44" max="44" width="12.8967012677874" customWidth="1" style="4"/>
-    <col min="45" max="45" width="12.7688184465681" customWidth="1" style="4"/>
-    <col min="46" max="46" width="12.8537325177874" customWidth="1" style="4"/>
-    <col min="47" max="47" width="12.7258496965681" customWidth="1" style="4"/>
-    <col min="48" max="48" width="13.4399490356445" customWidth="1" style="4"/>
-    <col min="49" max="49" width="13.3120662144252" customWidth="1" style="4"/>
-    <col min="50" max="50" width="13.3969802856445" customWidth="1" style="4"/>
-    <col min="51" max="51" width="13.2690974644252" customWidth="1" style="4"/>
-    <col min="52" max="52" width="10.0812247140067" customWidth="1" style="4"/>
-    <col min="53" max="53" width="9.95334189278739" customWidth="1" style="4"/>
-    <col min="54" max="54" width="10.300161089216" customWidth="1" style="4"/>
-    <col min="55" max="55" width="10.1722782679967" customWidth="1" style="4"/>
-    <col min="56" max="56" width="10.0812247140067" customWidth="1" style="4"/>
-    <col min="57" max="57" width="9.95334189278739" customWidth="1" style="4"/>
-    <col min="58" max="58" width="10.300161089216" customWidth="1" style="4"/>
-    <col min="59" max="59" width="10.1722782679967" customWidth="1" style="4"/>
-    <col min="60" max="60" width="10.0812247140067" customWidth="1" style="4"/>
-    <col min="61" max="61" width="9.95334189278739" customWidth="1" style="4"/>
-    <col min="62" max="62" width="10.300161089216" customWidth="1" style="4"/>
-    <col min="63" max="63" width="10.1722782679967" customWidth="1" style="4"/>
-    <col min="64" max="64" width="10.0812247140067" customWidth="1" style="4"/>
-    <col min="65" max="65" width="9.95334189278739" customWidth="1"/>
-    <col min="66" max="66" width="10.300161089216" customWidth="1"/>
-    <col min="67" max="67" width="10.1722782679967" customWidth="1"/>
-    <col min="68" max="68" width="10.0812247140067" customWidth="1"/>
-    <col min="69" max="69" width="9.95334189278739" customWidth="1"/>
-    <col min="70" max="70" width="10.300161089216" customWidth="1"/>
-    <col min="71" max="71" width="10.1722782679967" customWidth="1"/>
-    <col min="72" max="72" width="10.0812247140067" customWidth="1"/>
-    <col min="73" max="73" width="9.95334189278739" customWidth="1"/>
-    <col min="74" max="74" width="10.300161089216" customWidth="1"/>
-    <col min="75" max="75" width="10.1722782679967" customWidth="1"/>
-    <col min="76" max="76" width="10.0812247140067" customWidth="1"/>
-    <col min="77" max="77" width="9.95334189278739" customWidth="1"/>
-    <col min="78" max="78" width="10.300161089216" customWidth="1"/>
-    <col min="79" max="79" width="10.1722782679967" customWidth="1"/>
-    <col min="80" max="80" width="10.0812247140067" customWidth="1"/>
-    <col min="81" max="81" width="9.95334189278739" customWidth="1"/>
-    <col min="82" max="82" width="10.300161089216" customWidth="1"/>
-    <col min="83" max="83" width="10.1722782679967" customWidth="1"/>
-    <col min="84" max="84" width="10.0812247140067" customWidth="1"/>
-    <col min="85" max="85" width="9.95334189278739" customWidth="1"/>
-    <col min="86" max="86" width="10.300161089216" customWidth="1"/>
-    <col min="87" max="87" width="10.1722782679967" customWidth="1"/>
-    <col min="88" max="88" width="11.6761845179967" customWidth="1"/>
-    <col min="89" max="89" width="11.5483006068638" customWidth="1"/>
-    <col min="90" max="90" width="11.8951198032924" customWidth="1"/>
-    <col min="91" max="91" width="11.7672369820731" customWidth="1"/>
-    <col min="92" max="92" width="11.6761845179967" customWidth="1"/>
-    <col min="93" max="93" width="11.5483006068638" customWidth="1"/>
-    <col min="94" max="94" width="11.8951198032924" customWidth="1"/>
-    <col min="95" max="95" width="11.7672369820731" customWidth="1"/>
-    <col min="96" max="96" width="11.6761845179967" customWidth="1"/>
-    <col min="97" max="97" width="11.5483006068638" customWidth="1"/>
-    <col min="98" max="98" width="11.8951198032924" customWidth="1"/>
-    <col min="99" max="99" width="11.7672369820731" customWidth="1"/>
-    <col min="100" max="100" width="11.6761845179967" customWidth="1"/>
-    <col min="101" max="101" width="11.5483006068638" customWidth="1"/>
-    <col min="102" max="102" width="11.8951198032924" customWidth="1"/>
-    <col min="103" max="103" width="11.7672369820731" customWidth="1"/>
-    <col min="104" max="104" width="11.6761845179967" customWidth="1"/>
-    <col min="105" max="105" width="11.5483006068638" customWidth="1"/>
-    <col min="106" max="106" width="11.8951198032924" customWidth="1"/>
-    <col min="107" max="107" width="11.7672369820731" customWidth="1"/>
-    <col min="108" max="108" width="12.8465706961496" customWidth="1"/>
-    <col min="109" max="109" width="12.7186878749302" customWidth="1"/>
-    <col min="110" max="110" width="12.8465706961496" customWidth="1"/>
-    <col min="111" max="111" width="12.7186878749302" customWidth="1"/>
-    <col min="112" max="112" width="12.8465706961496" customWidth="1"/>
-    <col min="113" max="113" width="12.7186878749302" customWidth="1"/>
-    <col min="114" max="114" width="12.8465706961496" customWidth="1"/>
-    <col min="115" max="115" width="12.7186878749302" customWidth="1"/>
-    <col min="116" max="116" width="12.8465706961496" customWidth="1"/>
-    <col min="117" max="117" width="12.7186878749302" customWidth="1"/>
-    <col min="118" max="118" width="12.8465706961496" customWidth="1"/>
-    <col min="119" max="119" width="12.7186878749302" customWidth="1"/>
-    <col min="120" max="120" width="12.8465706961496" customWidth="1"/>
-    <col min="121" max="121" width="12.7186878749302" customWidth="1"/>
-    <col min="122" max="122" width="12.8465706961496" customWidth="1"/>
-    <col min="123" max="123" width="12.7186878749302" customWidth="1"/>
-    <col min="124" max="124" width="12.8465706961496" customWidth="1"/>
-    <col min="125" max="125" width="12.7186878749302" customWidth="1"/>
-    <col min="126" max="126" width="11.7406376429967" customWidth="1"/>
-    <col min="127" max="127" width="11.6127537318638" customWidth="1"/>
-    <col min="128" max="128" width="11.7406376429967" customWidth="1"/>
-    <col min="129" max="129" width="11.6127537318638" customWidth="1"/>
-    <col min="130" max="130" width="11.7406376429967" customWidth="1"/>
-    <col min="131" max="131" width="11.6127537318638" customWidth="1"/>
-    <col min="132" max="132" width="11.7406376429967" customWidth="1"/>
-    <col min="133" max="133" width="11.6127537318638" customWidth="1"/>
-    <col min="134" max="134" width="11.7406376429967" customWidth="1"/>
-    <col min="135" max="135" width="11.6127537318638" customWidth="1"/>
-    <col min="136" max="136" width="11.7406376429967" customWidth="1"/>
-    <col min="137" max="137" width="11.6127537318638" customWidth="1"/>
-    <col min="138" max="138" width="11.7406376429967" customWidth="1"/>
-    <col min="139" max="139" width="11.6127537318638" customWidth="1"/>
-    <col min="140" max="140" width="11.7406376429967" customWidth="1"/>
-    <col min="141" max="141" width="11.6127537318638" customWidth="1"/>
-    <col min="142" max="142" width="11.7406376429967" customWidth="1"/>
-    <col min="143" max="143" width="11.6127537318638" customWidth="1"/>
-    <col min="144" max="144" width="11.7406376429967" customWidth="1"/>
-    <col min="145" max="145" width="11.6127537318638" customWidth="1"/>
-    <col min="146" max="146" width="11.7406376429967" customWidth="1"/>
-    <col min="147" max="147" width="11.6127537318638" customWidth="1"/>
-    <col min="148" max="148" width="11.7406376429967" customWidth="1"/>
-    <col min="149" max="149" width="11.6127537318638" customWidth="1"/>
-    <col min="150" max="150" width="11.7406376429967" customWidth="1"/>
-    <col min="151" max="151" width="11.6127537318638" customWidth="1"/>
-    <col min="152" max="152" width="11.7406376429967" customWidth="1"/>
-    <col min="153" max="153" width="11.6127537318638" customWidth="1"/>
-    <col min="154" max="154" width="11.7406376429967" customWidth="1"/>
-    <col min="155" max="155" width="11.6127537318638" customWidth="1"/>
-    <col min="156" max="156" width="11.7406376429967" customWidth="1"/>
-    <col min="157" max="157" width="11.6127537318638" customWidth="1"/>
-    <col min="158" max="158" width="11.7406376429967" customWidth="1"/>
-    <col min="159" max="159" width="11.6127537318638" customWidth="1"/>
-    <col min="160" max="160" width="11.7406376429967" customWidth="1"/>
-    <col min="161" max="161" width="11.6127537318638" customWidth="1"/>
-    <col min="162" max="162" width="11.7406376429967" customWidth="1"/>
-    <col min="163" max="163" width="11.6127537318638" customWidth="1"/>
-    <col min="164" max="164" width="11.7406376429967" customWidth="1"/>
-    <col min="165" max="165" width="11.6127537318638" customWidth="1"/>
-    <col min="166" max="166" width="11.7406376429967" customWidth="1"/>
-    <col min="167" max="167" width="11.6127537318638" customWidth="1"/>
-    <col min="168" max="168" width="11.7406376429967" customWidth="1"/>
-    <col min="169" max="169" width="11.6127537318638" customWidth="1"/>
-    <col min="170" max="170" width="11.7406376429967" customWidth="1"/>
-    <col min="171" max="171" width="11.6127537318638" customWidth="1"/>
-    <col min="172" max="172" width="11.7406376429967" customWidth="1"/>
-    <col min="173" max="173" width="11.6127537318638" customWidth="1"/>
-    <col min="174" max="174" width="11.7406376429967" customWidth="1"/>
-    <col min="175" max="175" width="11.6127537318638" customWidth="1"/>
-    <col min="176" max="176" width="11.7406376429967" customWidth="1"/>
-    <col min="177" max="177" width="11.6127537318638" customWidth="1"/>
-    <col min="178" max="178" width="11.7406376429967" customWidth="1"/>
-    <col min="179" max="179" width="11.6127537318638" customWidth="1"/>
-    <col min="180" max="180" width="11.7406376429967" customWidth="1"/>
-    <col min="181" max="181" width="11.6127537318638" customWidth="1"/>
-    <col min="182" max="182" width="11.7406376429967" customWidth="1"/>
-    <col min="183" max="183" width="11.6127537318638" customWidth="1"/>
-    <col min="184" max="184" width="11.7406376429967" customWidth="1"/>
-    <col min="185" max="185" width="11.6127537318638" customWidth="1"/>
-    <col min="186" max="186" width="11.7406376429967" customWidth="1"/>
-    <col min="187" max="187" width="11.6127537318638" customWidth="1"/>
-    <col min="188" max="188" width="11.7406376429967" customWidth="1"/>
-    <col min="189" max="189" width="11.6127537318638" customWidth="1"/>
-    <col min="190" max="190" width="11.7406376429967" customWidth="1"/>
-    <col min="191" max="191" width="11.6127537318638" customWidth="1"/>
-    <col min="192" max="192" width="11.7406376429967" customWidth="1"/>
-    <col min="193" max="193" width="11.6127537318638" customWidth="1"/>
-    <col min="194" max="194" width="11.7406376429967" customWidth="1"/>
-    <col min="195" max="195" width="11.6127537318638" customWidth="1"/>
-    <col min="196" max="196" width="11.7406376429967" customWidth="1"/>
-    <col min="197" max="197" width="11.6127537318638" customWidth="1"/>
-    <col min="198" max="198" width="13.3355963570731" customWidth="1"/>
-    <col min="199" max="199" width="13.2077135358538" customWidth="1"/>
-    <col min="200" max="200" width="13.3355963570731" customWidth="1"/>
-    <col min="201" max="201" width="13.2077135358538" customWidth="1"/>
-    <col min="202" max="202" width="13.3355963570731" customWidth="1"/>
-    <col min="203" max="203" width="13.2077135358538" customWidth="1"/>
-    <col min="204" max="204" width="13.3355963570731" customWidth="1"/>
-    <col min="205" max="205" width="13.2077135358538" customWidth="1"/>
-    <col min="206" max="206" width="13.3355963570731" customWidth="1"/>
-    <col min="207" max="207" width="13.2077135358538" customWidth="1"/>
-    <col min="208" max="208" width="13.3355963570731" customWidth="1"/>
-    <col min="209" max="209" width="13.2077135358538" customWidth="1"/>
-    <col min="210" max="210" width="13.3355963570731" customWidth="1"/>
-    <col min="211" max="211" width="13.2077135358538" customWidth="1"/>
-    <col min="212" max="212" width="13.3355963570731" customWidth="1"/>
-    <col min="213" max="213" width="13.2077135358538" customWidth="1"/>
-    <col min="214" max="214" width="13.3355963570731" customWidth="1"/>
-    <col min="215" max="215" width="13.2077135358538" customWidth="1"/>
-    <col min="216" max="216" width="13.3355963570731" customWidth="1"/>
-    <col min="217" max="217" width="13.2077135358538" customWidth="1"/>
-    <col min="218" max="218" width="13.3355963570731" customWidth="1"/>
-    <col min="219" max="219" width="13.2077135358538" customWidth="1"/>
-    <col min="220" max="220" width="13.3355963570731" customWidth="1"/>
-    <col min="221" max="221" width="13.2077135358538" customWidth="1"/>
-    <col min="222" max="222" width="13.3355963570731" customWidth="1"/>
-    <col min="223" max="223" width="13.2077135358538" customWidth="1"/>
-    <col min="224" max="224" width="13.3355963570731" customWidth="1"/>
-    <col min="225" max="225" width="13.2077135358538" customWidth="1"/>
-    <col min="226" max="226" width="13.3355963570731" customWidth="1"/>
-    <col min="227" max="227" width="13.2077135358538" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="29.44140625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="25" style="4" customWidth="1"/>
+    <col min="7" max="7" width="19.21875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" style="4" customWidth="1"/>
+    <col min="9" max="9" width="13.77734375" style="4" customWidth="1"/>
+    <col min="10" max="33" width="9.109375" style="4" customWidth="1"/>
+    <col min="34" max="34" width="10.5546875" style="4" customWidth="1"/>
+    <col min="35" max="35" width="10.44140625" style="4" customWidth="1"/>
+    <col min="36" max="36" width="10.5546875" style="4" customWidth="1"/>
+    <col min="37" max="37" width="10.44140625" style="4" customWidth="1"/>
+    <col min="38" max="38" width="10.5546875" style="4" customWidth="1"/>
+    <col min="39" max="39" width="10.44140625" style="4" customWidth="1"/>
+    <col min="40" max="40" width="10.77734375" style="4" customWidth="1"/>
+    <col min="41" max="41" width="10.6640625" style="4" customWidth="1"/>
+    <col min="42" max="42" width="10.77734375" style="4" customWidth="1"/>
+    <col min="43" max="43" width="10.6640625" style="4" customWidth="1"/>
+    <col min="44" max="44" width="12.88671875" style="4" customWidth="1"/>
+    <col min="45" max="45" width="12.77734375" style="4" customWidth="1"/>
+    <col min="46" max="46" width="12.88671875" style="4" customWidth="1"/>
+    <col min="47" max="47" width="12.6640625" style="4" customWidth="1"/>
+    <col min="48" max="48" width="13.44140625" style="4" customWidth="1"/>
+    <col min="49" max="49" width="13.33203125" style="4" customWidth="1"/>
+    <col min="50" max="50" width="13.44140625" style="4" customWidth="1"/>
+    <col min="51" max="51" width="13.21875" style="4" customWidth="1"/>
+    <col min="52" max="52" width="10.109375" style="4" customWidth="1"/>
+    <col min="53" max="53" width="10" style="4" customWidth="1"/>
+    <col min="54" max="54" width="10.33203125" style="4" customWidth="1"/>
+    <col min="55" max="55" width="10.21875" style="4" customWidth="1"/>
+    <col min="56" max="56" width="10.109375" style="4" customWidth="1"/>
+    <col min="57" max="57" width="10" style="4" customWidth="1"/>
+    <col min="58" max="58" width="10.33203125" style="4" customWidth="1"/>
+    <col min="59" max="59" width="10.21875" style="4" customWidth="1"/>
+    <col min="60" max="60" width="10.109375" style="4" customWidth="1"/>
+    <col min="61" max="61" width="10" style="4" customWidth="1"/>
+    <col min="62" max="62" width="10.33203125" style="4" customWidth="1"/>
+    <col min="63" max="63" width="10.21875" style="4" customWidth="1"/>
+    <col min="64" max="64" width="10.109375" style="4" customWidth="1"/>
+    <col min="65" max="65" width="10" customWidth="1"/>
+    <col min="66" max="66" width="10.33203125" customWidth="1"/>
+    <col min="67" max="67" width="10.21875" customWidth="1"/>
+    <col min="68" max="68" width="10.109375" customWidth="1"/>
+    <col min="69" max="69" width="10" customWidth="1"/>
+    <col min="70" max="70" width="10.33203125" customWidth="1"/>
+    <col min="71" max="71" width="10.21875" customWidth="1"/>
+    <col min="72" max="72" width="10.109375" customWidth="1"/>
+    <col min="73" max="73" width="10" customWidth="1"/>
+    <col min="74" max="74" width="10.33203125" customWidth="1"/>
+    <col min="75" max="75" width="10.21875" customWidth="1"/>
+    <col min="76" max="76" width="10.109375" customWidth="1"/>
+    <col min="77" max="77" width="10" customWidth="1"/>
+    <col min="78" max="78" width="10.33203125" customWidth="1"/>
+    <col min="79" max="79" width="10.21875" customWidth="1"/>
+    <col min="80" max="80" width="10.109375" customWidth="1"/>
+    <col min="81" max="81" width="10" customWidth="1"/>
+    <col min="82" max="82" width="10.33203125" customWidth="1"/>
+    <col min="83" max="83" width="10.21875" customWidth="1"/>
+    <col min="84" max="84" width="10.109375" customWidth="1"/>
+    <col min="85" max="85" width="10" customWidth="1"/>
+    <col min="86" max="86" width="10.33203125" customWidth="1"/>
+    <col min="87" max="87" width="10.21875" customWidth="1"/>
+    <col min="88" max="88" width="11.6640625" customWidth="1"/>
+    <col min="89" max="89" width="11.5546875" customWidth="1"/>
+    <col min="90" max="90" width="11.88671875" customWidth="1"/>
+    <col min="91" max="91" width="11.77734375" customWidth="1"/>
+    <col min="92" max="92" width="11.6640625" customWidth="1"/>
+    <col min="93" max="93" width="11.5546875" customWidth="1"/>
+    <col min="94" max="94" width="11.88671875" customWidth="1"/>
+    <col min="95" max="95" width="11.77734375" customWidth="1"/>
+    <col min="96" max="96" width="11.6640625" customWidth="1"/>
+    <col min="97" max="97" width="11.5546875" customWidth="1"/>
+    <col min="98" max="98" width="11.88671875" customWidth="1"/>
+    <col min="99" max="99" width="11.77734375" customWidth="1"/>
+    <col min="100" max="100" width="11.6640625" customWidth="1"/>
+    <col min="101" max="101" width="11.5546875" customWidth="1"/>
+    <col min="102" max="102" width="11.88671875" customWidth="1"/>
+    <col min="103" max="103" width="11.77734375" customWidth="1"/>
+    <col min="104" max="104" width="11.6640625" customWidth="1"/>
+    <col min="105" max="105" width="11.5546875" customWidth="1"/>
+    <col min="106" max="106" width="11.88671875" customWidth="1"/>
+    <col min="107" max="107" width="11.77734375" customWidth="1"/>
+    <col min="108" max="108" width="12.88671875" customWidth="1"/>
+    <col min="109" max="109" width="12.6640625" customWidth="1"/>
+    <col min="110" max="110" width="12.88671875" customWidth="1"/>
+    <col min="111" max="111" width="12.6640625" customWidth="1"/>
+    <col min="112" max="112" width="12.88671875" customWidth="1"/>
+    <col min="113" max="113" width="12.6640625" customWidth="1"/>
+    <col min="114" max="114" width="12.88671875" customWidth="1"/>
+    <col min="115" max="115" width="12.6640625" customWidth="1"/>
+    <col min="116" max="116" width="12.88671875" customWidth="1"/>
+    <col min="117" max="117" width="12.6640625" customWidth="1"/>
+    <col min="118" max="118" width="12.88671875" customWidth="1"/>
+    <col min="119" max="119" width="12.6640625" customWidth="1"/>
+    <col min="120" max="120" width="12.88671875" customWidth="1"/>
+    <col min="121" max="121" width="12.6640625" customWidth="1"/>
+    <col min="122" max="122" width="12.88671875" customWidth="1"/>
+    <col min="123" max="123" width="12.6640625" customWidth="1"/>
+    <col min="124" max="124" width="12.88671875" customWidth="1"/>
+    <col min="125" max="125" width="12.6640625" customWidth="1"/>
+    <col min="126" max="126" width="11.77734375" customWidth="1"/>
+    <col min="127" max="127" width="11.5546875" customWidth="1"/>
+    <col min="128" max="128" width="11.77734375" customWidth="1"/>
+    <col min="129" max="129" width="11.5546875" customWidth="1"/>
+    <col min="130" max="130" width="11.77734375" customWidth="1"/>
+    <col min="131" max="131" width="11.5546875" customWidth="1"/>
+    <col min="132" max="132" width="11.77734375" customWidth="1"/>
+    <col min="133" max="133" width="11.5546875" customWidth="1"/>
+    <col min="134" max="134" width="11.77734375" customWidth="1"/>
+    <col min="135" max="135" width="11.5546875" customWidth="1"/>
+    <col min="136" max="136" width="11.77734375" customWidth="1"/>
+    <col min="137" max="137" width="11.5546875" customWidth="1"/>
+    <col min="138" max="138" width="11.77734375" customWidth="1"/>
+    <col min="139" max="139" width="11.5546875" customWidth="1"/>
+    <col min="140" max="140" width="11.77734375" customWidth="1"/>
+    <col min="141" max="141" width="11.5546875" customWidth="1"/>
+    <col min="142" max="142" width="11.77734375" customWidth="1"/>
+    <col min="143" max="143" width="11.5546875" customWidth="1"/>
+    <col min="144" max="144" width="11.77734375" customWidth="1"/>
+    <col min="145" max="145" width="11.5546875" customWidth="1"/>
+    <col min="146" max="146" width="11.77734375" customWidth="1"/>
+    <col min="147" max="147" width="11.5546875" customWidth="1"/>
+    <col min="148" max="148" width="11.77734375" customWidth="1"/>
+    <col min="149" max="149" width="11.5546875" customWidth="1"/>
+    <col min="150" max="150" width="11.77734375" customWidth="1"/>
+    <col min="151" max="151" width="11.5546875" customWidth="1"/>
+    <col min="152" max="152" width="11.77734375" customWidth="1"/>
+    <col min="153" max="153" width="11.5546875" customWidth="1"/>
+    <col min="154" max="154" width="11.77734375" customWidth="1"/>
+    <col min="155" max="155" width="11.5546875" customWidth="1"/>
+    <col min="156" max="156" width="11.77734375" customWidth="1"/>
+    <col min="157" max="157" width="11.5546875" customWidth="1"/>
+    <col min="158" max="158" width="11.77734375" customWidth="1"/>
+    <col min="159" max="159" width="11.5546875" customWidth="1"/>
+    <col min="160" max="160" width="11.77734375" customWidth="1"/>
+    <col min="161" max="161" width="11.5546875" customWidth="1"/>
+    <col min="162" max="162" width="11.77734375" customWidth="1"/>
+    <col min="163" max="163" width="11.5546875" customWidth="1"/>
+    <col min="164" max="164" width="11.77734375" customWidth="1"/>
+    <col min="165" max="165" width="11.5546875" customWidth="1"/>
+    <col min="166" max="166" width="11.77734375" customWidth="1"/>
+    <col min="167" max="167" width="11.5546875" customWidth="1"/>
+    <col min="168" max="168" width="11.77734375" customWidth="1"/>
+    <col min="169" max="169" width="11.5546875" customWidth="1"/>
+    <col min="170" max="170" width="11.77734375" customWidth="1"/>
+    <col min="171" max="171" width="11.5546875" customWidth="1"/>
+    <col min="172" max="172" width="11.77734375" customWidth="1"/>
+    <col min="173" max="173" width="11.5546875" customWidth="1"/>
+    <col min="174" max="174" width="11.77734375" customWidth="1"/>
+    <col min="175" max="175" width="11.5546875" customWidth="1"/>
+    <col min="176" max="176" width="11.77734375" customWidth="1"/>
+    <col min="177" max="177" width="11.5546875" customWidth="1"/>
+    <col min="178" max="178" width="11.77734375" customWidth="1"/>
+    <col min="179" max="179" width="11.5546875" customWidth="1"/>
+    <col min="180" max="180" width="11.77734375" customWidth="1"/>
+    <col min="181" max="181" width="11.5546875" customWidth="1"/>
+    <col min="182" max="182" width="11.77734375" customWidth="1"/>
+    <col min="183" max="183" width="11.5546875" customWidth="1"/>
+    <col min="184" max="184" width="11.77734375" customWidth="1"/>
+    <col min="185" max="185" width="11.5546875" customWidth="1"/>
+    <col min="186" max="186" width="11.77734375" customWidth="1"/>
+    <col min="187" max="187" width="11.5546875" customWidth="1"/>
+    <col min="188" max="188" width="11.77734375" customWidth="1"/>
+    <col min="189" max="189" width="11.5546875" customWidth="1"/>
+    <col min="190" max="190" width="11.77734375" customWidth="1"/>
+    <col min="191" max="191" width="11.5546875" customWidth="1"/>
+    <col min="192" max="192" width="11.77734375" customWidth="1"/>
+    <col min="193" max="193" width="11.5546875" customWidth="1"/>
+    <col min="194" max="194" width="11.77734375" customWidth="1"/>
+    <col min="195" max="195" width="11.5546875" customWidth="1"/>
+    <col min="196" max="196" width="11.77734375" customWidth="1"/>
+    <col min="197" max="197" width="11.5546875" customWidth="1"/>
+    <col min="198" max="198" width="13.33203125" customWidth="1"/>
+    <col min="199" max="199" width="13.21875" customWidth="1"/>
+    <col min="200" max="200" width="13.33203125" customWidth="1"/>
+    <col min="201" max="201" width="13.21875" customWidth="1"/>
+    <col min="202" max="202" width="13.33203125" customWidth="1"/>
+    <col min="203" max="203" width="13.21875" customWidth="1"/>
+    <col min="204" max="204" width="13.33203125" customWidth="1"/>
+    <col min="205" max="205" width="13.21875" customWidth="1"/>
+    <col min="206" max="206" width="13.33203125" customWidth="1"/>
+    <col min="207" max="207" width="13.21875" customWidth="1"/>
+    <col min="208" max="208" width="13.33203125" customWidth="1"/>
+    <col min="209" max="209" width="13.21875" customWidth="1"/>
+    <col min="210" max="210" width="13.33203125" customWidth="1"/>
+    <col min="211" max="211" width="13.21875" customWidth="1"/>
+    <col min="212" max="212" width="13.33203125" customWidth="1"/>
+    <col min="213" max="213" width="13.21875" customWidth="1"/>
+    <col min="214" max="214" width="13.33203125" customWidth="1"/>
+    <col min="215" max="215" width="13.21875" customWidth="1"/>
+    <col min="216" max="216" width="13.33203125" customWidth="1"/>
+    <col min="217" max="217" width="13.21875" customWidth="1"/>
+    <col min="218" max="218" width="13.33203125" customWidth="1"/>
+    <col min="219" max="219" width="13.21875" customWidth="1"/>
+    <col min="220" max="220" width="13.33203125" customWidth="1"/>
+    <col min="221" max="221" width="13.21875" customWidth="1"/>
+    <col min="222" max="222" width="13.33203125" customWidth="1"/>
+    <col min="223" max="223" width="13.21875" customWidth="1"/>
+    <col min="224" max="224" width="13.33203125" customWidth="1"/>
+    <col min="225" max="225" width="13.21875" customWidth="1"/>
+    <col min="226" max="226" width="13.33203125" customWidth="1"/>
+    <col min="227" max="227" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1818,667 +2071,667 @@
         <v>6</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="T1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="W1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="X1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="Y1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="Z1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="AA1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="AB1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AE1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AF1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AG1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="5" t="s">
+      <c r="AH1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AI1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AJ1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="5" t="s">
+      <c r="AK1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="5" t="s">
+      <c r="AL1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="5" t="s">
+      <c r="AM1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AN1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="5" t="s">
+      <c r="AO1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="5" t="s">
+      <c r="AP1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="5" t="s">
+      <c r="AQ1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="5" t="s">
+      <c r="AR1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="5" t="s">
+      <c r="AS1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="5" t="s">
+      <c r="AT1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="5" t="s">
+      <c r="AU1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="5" t="s">
+      <c r="AV1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="5" t="s">
+      <c r="AW1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="5" t="s">
+      <c r="AX1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" s="5" t="s">
+      <c r="AY1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="5" t="s">
+      <c r="AZ1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="5" t="s">
+      <c r="BA1" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" s="5" t="s">
+      <c r="BB1" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="5" t="s">
+      <c r="BC1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" s="5" t="s">
+      <c r="BD1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="5" t="s">
+      <c r="BE1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="5" t="s">
+      <c r="BF1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" s="5" t="s">
+      <c r="BG1" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" s="5" t="s">
+      <c r="BH1" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" s="5" t="s">
+      <c r="BI1" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" s="5" t="s">
+      <c r="BJ1" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" s="5" t="s">
+      <c r="BK1" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" s="5" t="s">
+      <c r="BL1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" s="5" t="s">
+      <c r="BM1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" s="5" t="s">
+      <c r="BN1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="BX1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="CB1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="CA1" s="1" t="s">
+      <c r="CC1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CD1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="CC1" s="1" t="s">
+      <c r="CE1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="CD1" s="1" t="s">
+      <c r="CF1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="CE1" s="1" t="s">
+      <c r="CG1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="CF1" s="1" t="s">
+      <c r="CH1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="CG1" s="1" t="s">
+      <c r="CI1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="CH1" s="1" t="s">
+      <c r="CJ1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="CI1" s="1" t="s">
+      <c r="CK1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="CJ1" s="1" t="s">
+      <c r="CL1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="CK1" s="1" t="s">
+      <c r="CM1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="CL1" s="1" t="s">
+      <c r="CN1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="CM1" s="1" t="s">
+      <c r="CO1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="CN1" s="1" t="s">
+      <c r="CP1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="CO1" s="1" t="s">
+      <c r="CQ1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="CP1" s="1" t="s">
+      <c r="CR1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="CQ1" s="1" t="s">
+      <c r="CS1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="CR1" s="1" t="s">
+      <c r="CT1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="CS1" s="1" t="s">
+      <c r="CU1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="CT1" s="1" t="s">
+      <c r="CV1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="CU1" s="1" t="s">
+      <c r="CW1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="CV1" s="1" t="s">
+      <c r="CX1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="CW1" s="1" t="s">
+      <c r="CY1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="CX1" s="1" t="s">
+      <c r="CZ1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="CY1" s="1" t="s">
+      <c r="DA1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="CZ1" s="1" t="s">
+      <c r="DB1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="DA1" s="1" t="s">
+      <c r="DC1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="DB1" s="1" t="s">
+      <c r="DD1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="DC1" s="1" t="s">
+      <c r="DE1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="DD1" s="1" t="s">
+      <c r="DF1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="DE1" s="1" t="s">
+      <c r="DG1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="DF1" s="1" t="s">
+      <c r="DH1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="DG1" s="1" t="s">
+      <c r="DI1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="DH1" s="1" t="s">
+      <c r="DJ1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="DI1" s="1" t="s">
+      <c r="DK1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="DJ1" s="1" t="s">
+      <c r="DL1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="DK1" s="1" t="s">
+      <c r="DM1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="DL1" s="1" t="s">
+      <c r="DN1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="DM1" s="1" t="s">
+      <c r="DO1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="DN1" s="1" t="s">
+      <c r="DP1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="DO1" s="1" t="s">
+      <c r="DQ1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="DP1" s="1" t="s">
+      <c r="DR1" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="DQ1" s="1" t="s">
+      <c r="DS1" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="DR1" s="1" t="s">
+      <c r="DT1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="DS1" s="1" t="s">
+      <c r="DU1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="DT1" s="1" t="s">
+      <c r="DV1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="DU1" s="1" t="s">
+      <c r="DW1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="DV1" s="1" t="s">
+      <c r="DX1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="DW1" s="1" t="s">
+      <c r="DY1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="DX1" s="1" t="s">
+      <c r="DZ1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="DY1" s="1" t="s">
+      <c r="EA1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="DZ1" s="1" t="s">
+      <c r="EB1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="EA1" s="1" t="s">
+      <c r="EC1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="EB1" s="1" t="s">
+      <c r="ED1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="EC1" s="1" t="s">
+      <c r="EE1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="ED1" s="1" t="s">
+      <c r="EF1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="EE1" s="1" t="s">
+      <c r="EG1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="EF1" s="1" t="s">
+      <c r="EH1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="EG1" s="1" t="s">
+      <c r="EI1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="EH1" s="1" t="s">
+      <c r="EJ1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="EI1" s="1" t="s">
+      <c r="EK1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="EJ1" s="1" t="s">
+      <c r="EL1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="EK1" s="1" t="s">
+      <c r="EM1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="EL1" s="1" t="s">
+      <c r="EN1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="EM1" s="1" t="s">
+      <c r="EO1" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="EN1" s="1" t="s">
+      <c r="EP1" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="EO1" s="1" t="s">
+      <c r="EQ1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="EP1" s="1" t="s">
+      <c r="ER1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="EQ1" s="1" t="s">
+      <c r="ES1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="ER1" s="1" t="s">
+      <c r="ET1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="ES1" s="1" t="s">
+      <c r="EU1" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="ET1" s="1" t="s">
+      <c r="EV1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="EU1" s="1" t="s">
+      <c r="EW1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="EV1" s="1" t="s">
+      <c r="EX1" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="EW1" s="1" t="s">
+      <c r="EY1" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="EX1" s="1" t="s">
+      <c r="EZ1" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="EY1" s="1" t="s">
+      <c r="FA1" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="EZ1" s="1" t="s">
+      <c r="FB1" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="FA1" s="1" t="s">
+      <c r="FC1" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="FB1" s="1" t="s">
+      <c r="FD1" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="FC1" s="1" t="s">
+      <c r="FE1" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="FD1" s="1" t="s">
+      <c r="FF1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="FE1" s="1" t="s">
+      <c r="FG1" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="FF1" s="1" t="s">
+      <c r="FH1" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="FG1" s="1" t="s">
+      <c r="FI1" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="FH1" s="1" t="s">
+      <c r="FJ1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="FI1" s="1" t="s">
+      <c r="FK1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="FJ1" s="1" t="s">
+      <c r="FL1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="FK1" s="1" t="s">
+      <c r="FM1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="FL1" s="1" t="s">
+      <c r="FN1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="FM1" s="1" t="s">
+      <c r="FO1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="FN1" s="1" t="s">
+      <c r="FP1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="FO1" s="1" t="s">
+      <c r="FQ1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="FP1" s="1" t="s">
+      <c r="FR1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="FQ1" s="1" t="s">
+      <c r="FS1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="FR1" s="1" t="s">
+      <c r="FT1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="FS1" s="1" t="s">
+      <c r="FU1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="FT1" s="1" t="s">
+      <c r="FV1" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="FU1" s="1" t="s">
+      <c r="FW1" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="FV1" s="1" t="s">
+      <c r="FX1" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="FW1" s="1" t="s">
+      <c r="FY1" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="FX1" s="1" t="s">
+      <c r="FZ1" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="FY1" s="1" t="s">
+      <c r="GA1" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="FZ1" s="1" t="s">
+      <c r="GB1" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="GA1" s="1" t="s">
+      <c r="GC1" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="GB1" s="1" t="s">
+      <c r="GD1" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="GC1" s="1" t="s">
+      <c r="GE1" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="GD1" s="1" t="s">
+      <c r="GF1" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="GE1" s="1" t="s">
+      <c r="GG1" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="GF1" s="1" t="s">
+      <c r="GH1" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="GG1" s="1" t="s">
+      <c r="GI1" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="GH1" s="1" t="s">
+      <c r="GJ1" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="GI1" s="1" t="s">
+      <c r="GK1" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="GJ1" s="1" t="s">
+      <c r="GL1" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="GK1" s="1" t="s">
+      <c r="GM1" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="GL1" s="1" t="s">
+      <c r="GN1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="GM1" s="1" t="s">
+      <c r="GO1" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="GN1" s="1" t="s">
+      <c r="GP1" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="GO1" s="1" t="s">
+      <c r="GQ1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="GP1" s="1" t="s">
+      <c r="GR1" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="GQ1" s="1" t="s">
+      <c r="GS1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="GR1" s="1" t="s">
+      <c r="GT1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="GS1" s="1" t="s">
+      <c r="GU1" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="GT1" s="1" t="s">
+      <c r="GV1" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="GU1" s="1" t="s">
+      <c r="GW1" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="GV1" s="1" t="s">
+      <c r="GX1" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="GW1" s="1" t="s">
+      <c r="GY1" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="GX1" s="1" t="s">
+      <c r="GZ1" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="GY1" s="1" t="s">
+      <c r="HA1" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="GZ1" s="1" t="s">
+      <c r="HB1" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="HA1" s="1" t="s">
+      <c r="HC1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="HB1" s="1" t="s">
+      <c r="HD1" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="HC1" s="1" t="s">
+      <c r="HE1" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="HD1" s="1" t="s">
+      <c r="HF1" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="HE1" s="1" t="s">
+      <c r="HG1" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="HF1" s="1" t="s">
+      <c r="HH1" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="HG1" s="1" t="s">
+      <c r="HI1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="HH1" s="1" t="s">
+      <c r="HJ1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="HI1" s="1" t="s">
+      <c r="HK1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="HJ1" s="1" t="s">
+      <c r="HL1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="HK1" s="1" t="s">
+      <c r="HM1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="HL1" s="1" t="s">
+      <c r="HN1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="HM1" s="1" t="s">
+      <c r="HO1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="HN1" s="1" t="s">
+      <c r="HP1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="HO1" s="1" t="s">
+      <c r="HQ1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="HP1" s="1" t="s">
+      <c r="HR1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="HQ1" s="1" t="s">
+      <c r="HS1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="HR1" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="HS1" s="1" t="s">
-        <v>226</v>
-      </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>64526</v>
       </c>
@@ -2486,43 +2739,43 @@
         <v>0</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E2" s="6">
+        <v>46078.958333333299</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="E2" s="6">
-        <v>46078.9583333333</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="H2" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="I2" s="7">
+        <v>2</v>
+      </c>
+      <c r="J2" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="K2" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="I2" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="M2" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="O2" s="9" t="s">
         <v>235</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>236</v>
-      </c>
-      <c r="O2" s="9" t="s">
-        <v>237</v>
       </c>
       <c r="P2" s="8"/>
       <c r="Q2" s="9"/>
@@ -2737,7 +2990,7 @@
       <c r="HR2" s="2"/>
       <c r="HS2" s="3"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>64527</v>
       </c>
@@ -2745,43 +2998,43 @@
         <v>0</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E3" s="6">
+        <v>46078.958333333299</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="E3" s="6">
-        <v>46078.9583333333</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="H3" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I3" s="7">
+        <v>2</v>
+      </c>
+      <c r="J3" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="K3" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="H3" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J3" s="8" t="s">
+      <c r="L3" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="M3" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="N3" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="L3" s="8" t="s">
-        <v>237</v>
-      </c>
-      <c r="M3" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>243</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="O3" s="9" t="s">
-        <v>245</v>
       </c>
       <c r="P3" s="8"/>
       <c r="Q3" s="9"/>
@@ -2996,7 +3249,7 @@
       <c r="HR3" s="2"/>
       <c r="HS3" s="3"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>64528</v>
       </c>
@@ -3004,43 +3257,43 @@
         <v>0</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E4" s="6">
+        <v>46078.958333333299</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="E4" s="6">
-        <v>46078.9583333333</v>
-      </c>
-      <c r="F4" s="4" t="s">
+      <c r="H4" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I4" s="7">
+        <v>2</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="K4" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="H4" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J4" s="8" t="s">
+      <c r="L4" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="N4" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>250</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="N4" s="8" t="s">
-        <v>251</v>
-      </c>
       <c r="O4" s="9" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="P4" s="8"/>
       <c r="Q4" s="9"/>
@@ -3255,7 +3508,7 @@
       <c r="HR4" s="2"/>
       <c r="HS4" s="3"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>64534</v>
       </c>
@@ -3263,43 +3516,43 @@
         <v>0</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="E5" s="6">
+        <v>46078.958333333299</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="E5" s="6">
-        <v>46078.9583333333</v>
-      </c>
-      <c r="F5" s="4" t="s">
+      <c r="H5" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="K5" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="M5" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="N5" s="8" t="s">
         <v>258</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="O5" s="9" t="s">
         <v>259</v>
-      </c>
-      <c r="N5" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="O5" s="9" t="s">
-        <v>261</v>
       </c>
       <c r="P5" s="8"/>
       <c r="Q5" s="9"/>
@@ -3514,7 +3767,7 @@
       <c r="HR5" s="2"/>
       <c r="HS5" s="3"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>64535</v>
       </c>
@@ -3522,43 +3775,43 @@
         <v>0</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="E6" s="6">
+        <v>46078.958333333299</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="E6" s="6">
-        <v>46078.9583333333</v>
-      </c>
-      <c r="F6" s="4" t="s">
+      <c r="H6" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="K6" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="L6" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K6" s="9" t="s">
+      <c r="M6" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="L6" s="8" t="s">
+      <c r="N6" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="M6" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="N6" s="8" t="s">
-        <v>268</v>
-      </c>
       <c r="O6" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="P6" s="8"/>
       <c r="Q6" s="9"/>
@@ -3773,7 +4026,7 @@
       <c r="HR6" s="2"/>
       <c r="HS6" s="3"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>64554</v>
       </c>
@@ -3781,43 +4034,43 @@
         <v>0</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="E7" s="6">
+        <v>46078.958333333299</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="E7" s="6">
-        <v>46078.9583333333</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="H7" s="7">
+        <v>1</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J7" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="K7" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="K7" s="9" t="s">
+      <c r="M7" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="N7" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="M7" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="N7" s="8" t="s">
-        <v>277</v>
-      </c>
       <c r="O7" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="P7" s="8"/>
       <c r="Q7" s="9"/>
@@ -4032,7 +4285,7 @@
       <c r="HR7" s="2"/>
       <c r="HS7" s="3"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>64551</v>
       </c>
@@ -4040,43 +4293,43 @@
         <v>0</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="E8" s="6">
+        <v>46078.947916666701</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="E8" s="6">
-        <v>46078.9479166667</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="H8" s="7">
+        <v>1</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="K8" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="L8" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="K8" s="9" t="s">
+      <c r="M8" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="N8" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="L8" s="8" t="s">
-        <v>282</v>
-      </c>
-      <c r="M8" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="N8" s="8" t="s">
-        <v>283</v>
-      </c>
       <c r="O8" s="9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="P8" s="8"/>
       <c r="Q8" s="9"/>
@@ -4291,7 +4544,7 @@
       <c r="HR8" s="2"/>
       <c r="HS8" s="3"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>64552</v>
       </c>
@@ -4299,43 +4552,43 @@
         <v>0</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="E9" s="6">
+        <v>46078.947916666701</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="E9" s="6">
-        <v>46078.9479166667</v>
-      </c>
-      <c r="F9" s="4" t="s">
+      <c r="H9" s="7">
+        <v>1</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J9" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="K9" s="9" t="s">
         <v>286</v>
       </c>
-      <c r="H9" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="M9" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="N9" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="M9" s="9" t="s">
+      <c r="O9" s="9" t="s">
         <v>290</v>
-      </c>
-      <c r="N9" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="O9" s="9" t="s">
-        <v>292</v>
       </c>
       <c r="P9" s="8"/>
       <c r="Q9" s="9"/>
@@ -4550,7 +4803,7 @@
       <c r="HR9" s="2"/>
       <c r="HS9" s="3"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>64553</v>
       </c>
@@ -4558,43 +4811,43 @@
         <v>0</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="E10" s="6">
+        <v>46078.947916666701</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="E10" s="6">
-        <v>46078.9479166667</v>
-      </c>
-      <c r="F10" s="4" t="s">
+      <c r="H10" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="K10" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="L10" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="M10" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="N10" s="8" t="s">
         <v>295</v>
       </c>
-      <c r="H10" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>296</v>
-      </c>
-      <c r="K10" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>276</v>
-      </c>
-      <c r="M10" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="N10" s="8" t="s">
-        <v>297</v>
-      </c>
       <c r="O10" s="9" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="P10" s="8"/>
       <c r="Q10" s="9"/>
@@ -4809,7 +5062,7 @@
       <c r="HR10" s="2"/>
       <c r="HS10" s="3"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>64571</v>
       </c>
@@ -4817,43 +5070,43 @@
         <v>0</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="E11" s="6">
+        <v>46078.947916666701</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="E11" s="6">
-        <v>46078.9479166667</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="H11" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="M11" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="N11" s="8" t="s">
         <v>300</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="O11" s="9" t="s">
         <v>301</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>259</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="L11" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="M11" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="N11" s="8" t="s">
-        <v>302</v>
-      </c>
-      <c r="O11" s="9" t="s">
-        <v>303</v>
       </c>
       <c r="P11" s="8"/>
       <c r="Q11" s="9"/>
@@ -5068,7 +5321,7 @@
       <c r="HR11" s="2"/>
       <c r="HS11" s="3"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>64542</v>
       </c>
@@ -5076,43 +5329,43 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E12" s="6">
+        <v>46078.916666666701</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>305</v>
       </c>
-      <c r="E12" s="6">
-        <v>46078.9166666667</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="H12" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="L12" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="G12" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="K12" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="L12" s="8" t="s">
-        <v>308</v>
-      </c>
       <c r="M12" s="9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="N12" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="O12" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="P12" s="8"/>
       <c r="Q12" s="9"/>
@@ -5327,7 +5580,7 @@
       <c r="HR12" s="2"/>
       <c r="HS12" s="3"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>64562</v>
       </c>
@@ -5335,43 +5588,43 @@
         <v>0</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="E13" s="6">
+        <v>46078.916666666701</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>310</v>
       </c>
-      <c r="E13" s="6">
-        <v>46078.9166666667</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="H13" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="M13" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="N13" s="8" t="s">
         <v>311</v>
       </c>
-      <c r="G13" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>259</v>
-      </c>
-      <c r="K13" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="M13" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="N13" s="8" t="s">
-        <v>313</v>
-      </c>
       <c r="O13" s="9" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="P13" s="8"/>
       <c r="Q13" s="9"/>
@@ -5586,7 +5839,7 @@
       <c r="HR13" s="2"/>
       <c r="HS13" s="3"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>64563</v>
       </c>
@@ -5594,43 +5847,43 @@
         <v>0</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="E14" s="6">
+        <v>46078.916666666701</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="E14" s="6">
-        <v>46078.9166666667</v>
-      </c>
-      <c r="F14" s="4" t="s">
+      <c r="H14" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J14" s="8" t="s">
         <v>315</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="K14" s="9" t="s">
         <v>316</v>
       </c>
-      <c r="H14" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J14" s="8" t="s">
+      <c r="L14" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="M14" s="9" t="s">
         <v>317</v>
       </c>
-      <c r="K14" s="9" t="s">
+      <c r="N14" s="8" t="s">
         <v>318</v>
       </c>
-      <c r="L14" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="M14" s="9" t="s">
+      <c r="O14" s="9" t="s">
         <v>319</v>
-      </c>
-      <c r="N14" s="8" t="s">
-        <v>320</v>
-      </c>
-      <c r="O14" s="9" t="s">
-        <v>321</v>
       </c>
       <c r="P14" s="8"/>
       <c r="Q14" s="9"/>
@@ -5845,7 +6098,7 @@
       <c r="HR14" s="2"/>
       <c r="HS14" s="3"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>64540</v>
       </c>
@@ -5853,43 +6106,43 @@
         <v>0</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E15" s="6">
+        <v>46078.895833333299</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="E15" s="6">
-        <v>46078.8958333333</v>
-      </c>
-      <c r="F15" s="4" t="s">
+      <c r="H15" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="L15" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="M15" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="N15" s="8" t="s">
         <v>323</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="O15" s="9" t="s">
         <v>324</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="K15" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="L15" s="8" t="s">
-        <v>275</v>
-      </c>
-      <c r="M15" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="N15" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="O15" s="9" t="s">
-        <v>326</v>
       </c>
       <c r="P15" s="8"/>
       <c r="Q15" s="9"/>
@@ -6104,7 +6357,7 @@
       <c r="HR15" s="2"/>
       <c r="HS15" s="3"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>64541</v>
       </c>
@@ -6112,43 +6365,43 @@
         <v>0</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E16" s="6">
+        <v>46078.895833333299</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="E16" s="6">
-        <v>46078.8958333333</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>329</v>
-      </c>
       <c r="H16" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="M16" s="9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="O16" s="9" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="P16" s="8"/>
       <c r="Q16" s="9"/>
@@ -6363,7 +6616,7 @@
       <c r="HR16" s="2"/>
       <c r="HS16" s="3"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>64572</v>
       </c>
@@ -6371,43 +6624,43 @@
         <v>0</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="E17" s="6">
         <v>46078.875</v>
       </c>
       <c r="F17" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="H17" s="7">
+        <v>1</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="L17" s="8" t="s">
         <v>332</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="M17" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="N17" s="8" t="s">
         <v>333</v>
       </c>
-      <c r="H17" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>237</v>
-      </c>
-      <c r="K17" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="L17" s="8" t="s">
+      <c r="O17" s="9" t="s">
         <v>334</v>
-      </c>
-      <c r="M17" s="9" t="s">
-        <v>289</v>
-      </c>
-      <c r="N17" s="8" t="s">
-        <v>335</v>
-      </c>
-      <c r="O17" s="9" t="s">
-        <v>336</v>
       </c>
       <c r="P17" s="8"/>
       <c r="Q17" s="9"/>
@@ -6622,7 +6875,7 @@
       <c r="HR17" s="2"/>
       <c r="HS17" s="3"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>64573</v>
       </c>
@@ -6630,43 +6883,43 @@
         <v>0</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="E18" s="6">
         <v>46078.875</v>
       </c>
       <c r="F18" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="K18" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="M18" s="9" t="s">
         <v>339</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>340</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="K18" s="9" t="s">
-        <v>266</v>
-      </c>
-      <c r="L18" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="M18" s="9" t="s">
-        <v>341</v>
-      </c>
       <c r="N18" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="O18" s="9" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="P18" s="8"/>
       <c r="Q18" s="9"/>
@@ -6881,7 +7134,7 @@
       <c r="HR18" s="2"/>
       <c r="HS18" s="3"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>64525</v>
       </c>
@@ -6889,43 +7142,43 @@
         <v>0</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" s="6">
+        <v>46078.864583333299</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="E19" s="6">
-        <v>46078.8645833333</v>
-      </c>
-      <c r="F19" s="4" t="s">
+      <c r="H19" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I19" s="7">
+        <v>2</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="K19" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="G19" s="4" t="s">
-        <v>344</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>267</v>
-      </c>
-      <c r="K19" s="9" t="s">
-        <v>345</v>
-      </c>
       <c r="L19" s="8" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="N19" s="8" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="P19" s="8"/>
       <c r="Q19" s="9"/>
@@ -7140,7 +7393,7 @@
       <c r="HR19" s="2"/>
       <c r="HS19" s="3"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>64561</v>
       </c>
@@ -7148,43 +7401,43 @@
         <v>0</v>
       </c>
       <c r="C20" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="E20" s="6">
+        <v>46078.458333333299</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>346</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="G20" s="4" t="s">
         <v>347</v>
       </c>
-      <c r="E20" s="6">
-        <v>46078.4583333333</v>
-      </c>
-      <c r="F20" s="4" t="s">
+      <c r="H20" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J20" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="G20" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J20" s="8" t="s">
-        <v>350</v>
-      </c>
       <c r="K20" s="9" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="M20" s="9" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="O20" s="9" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="P20" s="8"/>
       <c r="Q20" s="9"/>
@@ -7399,7 +7652,7 @@
       <c r="HR20" s="2"/>
       <c r="HS20" s="3"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>64560</v>
       </c>
@@ -7407,43 +7660,43 @@
         <v>0</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E21" s="6">
         <v>46078.25</v>
       </c>
       <c r="F21" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J21" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="G21" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I21" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>355</v>
-      </c>
       <c r="K21" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="L21" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M21" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="L21" s="8" t="s">
-        <v>251</v>
-      </c>
-      <c r="M21" s="9" t="s">
-        <v>290</v>
-      </c>
       <c r="N21" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="P21" s="8"/>
       <c r="Q21" s="9"/>
@@ -7658,7 +7911,7 @@
       <c r="HR21" s="2"/>
       <c r="HS21" s="3"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>64533</v>
       </c>
@@ -7666,43 +7919,43 @@
         <v>0</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="E22" s="6">
+        <v>46078.166666666701</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>356</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="E22" s="6">
-        <v>46078.1666666667</v>
-      </c>
-      <c r="F22" s="4" t="s">
+      <c r="H22" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J22" s="8" t="s">
         <v>357</v>
       </c>
-      <c r="G22" s="4" t="s">
-        <v>358</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J22" s="8" t="s">
-        <v>359</v>
-      </c>
       <c r="K22" s="9" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="L22" s="8" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="M22" s="9" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="N22" s="8" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="O22" s="9" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="P22" s="8"/>
       <c r="Q22" s="9"/>
@@ -7917,7 +8170,7 @@
       <c r="HR22" s="2"/>
       <c r="HS22" s="3"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>64559</v>
       </c>
@@ -7925,43 +8178,43 @@
         <v>0</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E23" s="6">
+        <v>46078.166666666701</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>360</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="E23" s="6">
-        <v>46078.1666666667</v>
-      </c>
-      <c r="F23" s="4" t="s">
+      <c r="H23" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J23" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="G23" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J23" s="8" t="s">
-        <v>363</v>
-      </c>
       <c r="K23" s="9" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="L23" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="M23" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="N23" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="O23" s="9" t="s">
         <v>243</v>
-      </c>
-      <c r="M23" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="N23" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="O23" s="9" t="s">
-        <v>245</v>
       </c>
       <c r="P23" s="8"/>
       <c r="Q23" s="9"/>
@@ -8176,7 +8429,7 @@
       <c r="HR23" s="2"/>
       <c r="HS23" s="3"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>64532</v>
       </c>
@@ -8184,43 +8437,43 @@
         <v>0</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="E24" s="6">
+        <v>46078.145833333299</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="G24" s="4" t="s">
         <v>364</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="E24" s="6">
-        <v>46078.1458333333</v>
-      </c>
-      <c r="F24" s="4" t="s">
+      <c r="H24" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J24" s="8" t="s">
         <v>365</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="K24" s="9" t="s">
         <v>366</v>
       </c>
-      <c r="H24" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J24" s="8" t="s">
-        <v>367</v>
-      </c>
-      <c r="K24" s="9" t="s">
-        <v>368</v>
-      </c>
       <c r="L24" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="M24" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="N24" s="8" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="O24" s="9" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="P24" s="8"/>
       <c r="Q24" s="9"/>
@@ -8435,7 +8688,7 @@
       <c r="HR24" s="2"/>
       <c r="HS24" s="3"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>64538</v>
       </c>
@@ -8443,43 +8696,43 @@
         <v>0</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E25" s="6">
+        <v>46078.145833333299</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="E25" s="6">
-        <v>46078.1458333333</v>
-      </c>
-      <c r="F25" s="4" t="s">
+      <c r="H25" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J25" s="8" t="s">
         <v>370</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="K25" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="M25" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="N25" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="O25" s="9" t="s">
         <v>371</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>372</v>
-      </c>
-      <c r="K25" s="9" t="s">
-        <v>372</v>
-      </c>
-      <c r="L25" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="M25" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="N25" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="O25" s="9" t="s">
-        <v>373</v>
       </c>
       <c r="P25" s="8"/>
       <c r="Q25" s="9"/>
@@ -8694,7 +8947,7 @@
       <c r="HR25" s="2"/>
       <c r="HS25" s="3"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>64539</v>
       </c>
@@ -8702,43 +8955,43 @@
         <v>0</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E26" s="6">
+        <v>46078.145833333299</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="G26" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="E26" s="6">
-        <v>46078.1458333333</v>
-      </c>
-      <c r="F26" s="4" t="s">
+      <c r="H26" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J26" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="K26" s="9" t="s">
         <v>376</v>
       </c>
-      <c r="H26" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J26" s="8" t="s">
+      <c r="L26" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="M26" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="N26" s="8" t="s">
         <v>377</v>
       </c>
-      <c r="K26" s="9" t="s">
-        <v>378</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>237</v>
-      </c>
-      <c r="M26" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="N26" s="8" t="s">
-        <v>379</v>
-      </c>
       <c r="O26" s="9" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="P26" s="8"/>
       <c r="Q26" s="9"/>
@@ -8953,7 +9206,7 @@
       <c r="HR26" s="2"/>
       <c r="HS26" s="3"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>64575</v>
       </c>
@@ -8961,43 +9214,43 @@
         <v>0</v>
       </c>
       <c r="C27" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="E27" s="6">
+        <v>46078.145833333299</v>
+      </c>
+      <c r="F27" s="4" t="s">
         <v>380</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="G27" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="E27" s="6">
-        <v>46078.1458333333</v>
-      </c>
-      <c r="F27" s="4" t="s">
+      <c r="H27" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="K27" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="M27" s="9" t="s">
         <v>382</v>
       </c>
-      <c r="G27" s="4" t="s">
-        <v>383</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>297</v>
-      </c>
-      <c r="K27" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="L27" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="M27" s="9" t="s">
-        <v>384</v>
-      </c>
       <c r="N27" s="8" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="P27" s="8"/>
       <c r="Q27" s="9"/>
@@ -9212,7 +9465,7 @@
       <c r="HR27" s="2"/>
       <c r="HS27" s="3"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>64576</v>
       </c>
@@ -9220,43 +9473,43 @@
         <v>0</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="E28" s="6">
+        <v>46078.145833333299</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="G28" s="4" t="s">
         <v>385</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>381</v>
-      </c>
-      <c r="E28" s="6">
-        <v>46078.1458333333</v>
-      </c>
-      <c r="F28" s="4" t="s">
+      <c r="H28" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J28" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="K28" s="9" t="s">
         <v>387</v>
       </c>
-      <c r="H28" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I28" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J28" s="8" t="s">
+      <c r="L28" s="8" t="s">
         <v>388</v>
       </c>
-      <c r="K28" s="9" t="s">
+      <c r="M28" s="9" t="s">
+        <v>382</v>
+      </c>
+      <c r="N28" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="L28" s="8" t="s">
-        <v>390</v>
-      </c>
-      <c r="M28" s="9" t="s">
-        <v>384</v>
-      </c>
-      <c r="N28" s="8" t="s">
-        <v>391</v>
-      </c>
       <c r="O28" s="9" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="P28" s="8"/>
       <c r="Q28" s="9"/>
@@ -9471,7 +9724,7 @@
       <c r="HR28" s="2"/>
       <c r="HS28" s="3"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>64531</v>
       </c>
@@ -9479,43 +9732,43 @@
         <v>0</v>
       </c>
       <c r="C29" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="E29" s="6">
+        <v>46078.072916666701</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="D29" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="E29" s="6">
-        <v>46078.0729166667</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>393</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>394</v>
-      </c>
       <c r="H29" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="L29" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="M29" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="N29" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="O29" s="9" t="s">
         <v>259</v>
-      </c>
-      <c r="N29" s="8" t="s">
-        <v>283</v>
-      </c>
-      <c r="O29" s="9" t="s">
-        <v>261</v>
       </c>
       <c r="P29" s="8"/>
       <c r="Q29" s="9"/>
@@ -9730,7 +9983,7 @@
       <c r="HR29" s="2"/>
       <c r="HS29" s="3"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>64530</v>
       </c>
@@ -9738,43 +9991,43 @@
         <v>0</v>
       </c>
       <c r="C30" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="E30" s="6">
+        <v>46078.052083333299</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="G30" s="4" t="s">
         <v>395</v>
       </c>
-      <c r="D30" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="E30" s="6">
-        <v>46078.0520833333</v>
-      </c>
-      <c r="F30" s="4" t="s">
+      <c r="H30" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="K30" s="9" t="s">
         <v>396</v>
       </c>
-      <c r="G30" s="4" t="s">
-        <v>397</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J30" s="8" t="s">
-        <v>345</v>
-      </c>
-      <c r="K30" s="9" t="s">
-        <v>398</v>
-      </c>
       <c r="L30" s="8" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="M30" s="9" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="N30" s="8" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="O30" s="9" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="P30" s="8"/>
       <c r="Q30" s="9"/>
@@ -9989,7 +10242,7 @@
       <c r="HR30" s="2"/>
       <c r="HS30" s="3"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>64537</v>
       </c>
@@ -9997,43 +10250,43 @@
         <v>0</v>
       </c>
       <c r="C31" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E31" s="6">
+        <v>46078.041666666701</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="G31" s="4" t="s">
         <v>399</v>
       </c>
-      <c r="D31" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="E31" s="6">
-        <v>46078.0416666667</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>400</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>401</v>
-      </c>
       <c r="H31" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="L31" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="M31" s="9" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="N31" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="P31" s="8"/>
       <c r="Q31" s="9"/>
@@ -10248,7 +10501,7 @@
       <c r="HR31" s="2"/>
       <c r="HS31" s="3"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:227" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>64574</v>
       </c>
@@ -10256,43 +10509,43 @@
         <v>0</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="E32" s="6">
+        <v>46078.041666666701</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="G32" s="4" t="s">
         <v>402</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>381</v>
-      </c>
-      <c r="E32" s="6">
-        <v>46078.0416666667</v>
-      </c>
-      <c r="F32" s="4" t="s">
+      <c r="H32" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="J32" s="8" t="s">
         <v>403</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="K32" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="L32" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="M32" s="9" t="s">
         <v>404</v>
       </c>
-      <c r="H32" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J32" s="8" t="s">
-        <v>405</v>
-      </c>
-      <c r="K32" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="L32" s="8" t="s">
-        <v>265</v>
-      </c>
-      <c r="M32" s="9" t="s">
-        <v>406</v>
-      </c>
       <c r="N32" s="8" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="O32" s="9" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="P32" s="8"/>
       <c r="Q32" s="9"/>
@@ -10508,8 +10761,8 @@
       <c r="HS32" s="3"/>
     </row>
   </sheetData>
-  <headerFooter/>
-  <tableParts>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>

</xml_diff>